<commit_message>
fix: default optional player categories
</commit_message>
<xml_diff>
--- a/public/templates/player-import-template.xlsx
+++ b/public/templates/player-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="1" r:id="Ra3f5d6a06c9042f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R6faba87b698d4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="1" r:id="Rcb3dc230a32a46c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rb0a7da06b57e415c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -761,7 +761,7 @@
   </x:sheetData>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B501">
-      <x:formula1>"Batsman,Bowler,All-Rounder,Wicket-Keeper"</x:formula1>
+      <x:formula1>"Uncategorized,Batsman,Bowler,All-Rounder,Wicket-Keeper"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="D2:D501">
       <x:formula1>1000</x:formula1>
@@ -798,7 +798,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="25" t="str">
-        <x:v>Fill the Players sheet and upload the saved .xlsx file from Player Pool. Keep the header row unchanged.</x:v>
+        <x:v>Only Name and Base Price are required. Fill the Players sheet and upload the saved .xlsx file from Player Pool. Keep the header row unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -823,15 +823,15 @@
         <x:v>2–100 characters</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="63" t="str">
         <x:v>Category</x:v>
       </x:c>
       <x:c r="B7" s="53" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="C7" s="64" t="str">
-        <x:v>Batsman, Bowler, All-Rounder, or Wicket-Keeper</x:v>
+        <x:v>Leave blank to use Uncategorized, or choose Batsman, Bowler, All-Rounder, or Wicket-Keeper</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -842,7 +842,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="C8" s="64" t="str">
-        <x:v>Use a specialization that belongs to the selected category</x:v>
+        <x:v>Choose only when a category is selected</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">

</xml_diff>